<commit_message>
Migrate from Authentik to Keycloak and update Wazuh to Cloud API with provided key
</commit_message>
<xml_diff>
--- a/ELITE_HR_Master_Dashboard.xlsx
+++ b/ELITE_HR_Master_Dashboard.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offboarded Resources" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SecOps_Wazuh" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SecOps_Wazuh_DLP" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SecOps_Authentik" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SecOps_Keycloak" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CALC" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_CONTEXT" sheetId="14" state="visible" r:id="rId14"/>
@@ -529,7 +529,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,16 +538,16 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>44468</v>
+        <v>44272</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Manager B</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Under Probation</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -583,16 +583,16 @@
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>43998</v>
+        <v>44979</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Manager B</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Under Probation</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -628,16 +628,16 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>44824</v>
+        <v>43941</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager C</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Under Probation</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -673,16 +673,16 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>44500</v>
+        <v>44467</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Manager B</t>
+          <t>Manager C</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Under Probation</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>44137</v>
+        <v>45190</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -763,11 +763,11 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>45267</v>
+        <v>45225</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager C</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -808,16 +808,16 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>44781</v>
+        <v>44578</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager C</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -853,11 +853,11 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>44774</v>
+        <v>44631</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Manager B</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -898,16 +898,16 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>43944</v>
+        <v>45150</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Manager C</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>Under Probation</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -943,16 +943,16 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>44157</v>
+        <v>44020</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager C</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Under Probation</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -988,11 +988,11 @@
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>45290</v>
+        <v>44957</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Manager B</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1033,16 +1033,16 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>44846</v>
+        <v>44703</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>44564</v>
+        <v>45185</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1123,11 +1123,11 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>44037</v>
+        <v>45091</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Manager C</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1168,16 +1168,16 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>43928</v>
+        <v>43993</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Manager C</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Under Probation</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1213,16 +1213,16 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>45010</v>
+        <v>44998</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Under Probation</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>44684</v>
+        <v>43999</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Under Probation</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1303,11 +1303,11 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>45277</v>
+        <v>44610</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>43978</v>
+        <v>44831</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Under Probation</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1393,11 +1393,11 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>44613</v>
+        <v>44446</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Manager C</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>44526</v>
+        <v>43955</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1483,11 +1483,11 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>44562</v>
+        <v>44574</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Manager B</t>
+          <t>Manager C</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>43997</v>
+        <v>45069</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>44790</v>
+        <v>44857</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Under Probation</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1618,11 +1618,11 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>44263</v>
+        <v>45131</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Manager C</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1663,16 +1663,16 @@
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>45245</v>
+        <v>45007</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Under Probation</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1708,11 +1708,11 @@
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>44443</v>
+        <v>45167</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Manager C</t>
+          <t>Manager A</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1753,11 +1753,11 @@
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>44460</v>
+        <v>44901</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Manager A</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1798,7 +1798,7 @@
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>44406</v>
+        <v>44882</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1843,11 +1843,11 @@
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>45230</v>
+        <v>44038</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Manager C</t>
+          <t>Manager B</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>43787</v>
+        <v>44759</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>44423</v>
+        <v>44156</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>44250</v>
+        <v>43375</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>44061</v>
+        <v>43896</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>43603</v>
+        <v>43477</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>43965</v>
+        <v>44131</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>44392</v>
+        <v>44618</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>44731</v>
+        <v>43398</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>43188</v>
+        <v>43640</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>43584</v>
+        <v>44783</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1017639</v>
+        <v>2761037</v>
       </c>
     </row>
     <row r="3">
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1004629</v>
+        <v>1704789</v>
       </c>
     </row>
     <row r="4">
@@ -2475,7 +2475,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2453557</v>
+        <v>1773729</v>
       </c>
     </row>
     <row r="5">
@@ -2490,7 +2490,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1790693</v>
+        <v>608314</v>
       </c>
     </row>
     <row r="6">
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>990492</v>
+        <v>2015665</v>
       </c>
     </row>
     <row r="7">
@@ -2520,7 +2520,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1930977</v>
+        <v>1089923</v>
       </c>
     </row>
     <row r="8">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1321312</v>
+        <v>2338060</v>
       </c>
     </row>
     <row r="9">
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2970144</v>
+        <v>1477550</v>
       </c>
     </row>
     <row r="10">
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1636543</v>
+        <v>1072981</v>
       </c>
     </row>
     <row r="11">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>681011</v>
+        <v>1849980</v>
       </c>
     </row>
     <row r="12">
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1263672</v>
+        <v>2186985</v>
       </c>
     </row>
     <row r="13">
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>612668</v>
+        <v>2362776</v>
       </c>
     </row>
     <row r="14">
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1652049</v>
+        <v>810586</v>
       </c>
     </row>
     <row r="15">
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>654474</v>
+        <v>2781113</v>
       </c>
     </row>
     <row r="16">
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1993973</v>
+        <v>745858</v>
       </c>
     </row>
     <row r="17">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1149790</v>
+        <v>1215703</v>
       </c>
     </row>
     <row r="18">
@@ -2685,7 +2685,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1705268</v>
+        <v>2366153</v>
       </c>
     </row>
     <row r="19">
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>958306</v>
+        <v>2894004</v>
       </c>
     </row>
     <row r="20">
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2079053</v>
+        <v>2080386</v>
       </c>
     </row>
     <row r="21">
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1084773</v>
+        <v>1465190</v>
       </c>
     </row>
     <row r="22">
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1501334</v>
+        <v>2927440</v>
       </c>
     </row>
     <row r="23">
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1461738</v>
+        <v>1917657</v>
       </c>
     </row>
     <row r="24">
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1241917</v>
+        <v>1577921</v>
       </c>
     </row>
     <row r="25">
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1969564</v>
+        <v>2429841</v>
       </c>
     </row>
     <row r="26">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2155082</v>
+        <v>2082240</v>
       </c>
     </row>
     <row r="27">
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1528068</v>
+        <v>2256610</v>
       </c>
     </row>
     <row r="28">
@@ -2835,7 +2835,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2351424</v>
+        <v>2874687</v>
       </c>
     </row>
     <row r="29">
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1250459</v>
+        <v>1050509</v>
       </c>
     </row>
     <row r="30">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2619351</v>
+        <v>2620142</v>
       </c>
     </row>
     <row r="31">
@@ -2880,7 +2880,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>642580</v>
+        <v>756465</v>
       </c>
     </row>
     <row r="32">
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>154339</v>
+        <v>149324</v>
       </c>
     </row>
     <row r="33">
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>126921</v>
+        <v>165462</v>
       </c>
     </row>
     <row r="34">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>157391</v>
+        <v>126298</v>
       </c>
     </row>
     <row r="35">
@@ -2940,7 +2940,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>131013</v>
+        <v>84066</v>
       </c>
     </row>
     <row r="36">
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>142624</v>
+        <v>171712</v>
       </c>
     </row>
     <row r="37">
@@ -2970,7 +2970,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>179714</v>
+        <v>122930</v>
       </c>
     </row>
     <row r="38">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>115012</v>
+        <v>125905</v>
       </c>
     </row>
     <row r="39">
@@ -3000,7 +3000,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>93033</v>
+        <v>121422</v>
       </c>
     </row>
     <row r="40">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>114294</v>
+        <v>147033</v>
       </c>
     </row>
     <row r="41">
@@ -3030,7 +3030,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>127883</v>
+        <v>89257</v>
       </c>
     </row>
   </sheetData>
@@ -3076,11 +3076,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.864074340676935</v>
+        <v>8.990786705405309</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8.005185064029201</v>
+        <v>9.194512433738842</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8.67101840561253</v>
+        <v>8.176521034034051</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3121,11 +3121,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.576544639844474</v>
+        <v>8.900250238993422</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9.248183157742751</v>
+        <v>8.284085883202923</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.810490615165676</v>
+        <v>6.602700438511552</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3166,11 +3166,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8.689764313308201</v>
+        <v>7.406156717232985</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7.555887588138125</v>
+        <v>6.534235971063206</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8.796910564827295</v>
+        <v>8.229416671405746</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8.112161262889156</v>
+        <v>9.120797555806391</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -3226,11 +3226,11 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.277748460178811</v>
+        <v>7.003885324277586</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3241,11 +3241,11 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.814065369239937</v>
+        <v>9.490712404977797</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3256,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.883238490313608</v>
+        <v>7.400618734169834</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -3271,11 +3271,11 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8.515293664012709</v>
+        <v>7.389087906830456</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3286,11 +3286,11 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8.331071899877573</v>
+        <v>7.547324837200071</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8.478442064631441</v>
+        <v>8.106974865176198</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6.769803173394106</v>
+        <v>6.568305279067194</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -3331,7 +3331,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>8.420190905651657</v>
+        <v>8.548552549353442</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -3346,11 +3346,11 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6.719493305030126</v>
+        <v>8.521096663878456</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3361,11 +3361,11 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7.838856910960281</v>
+        <v>8.985863217611232</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>7.43738252001499</v>
+        <v>6.640887008553854</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>8.557141159677197</v>
+        <v>8.481043463391632</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -3406,11 +3406,11 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8.842509123520879</v>
+        <v>7.239443660678409</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3421,11 +3421,11 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6.956448323265212</v>
+        <v>8.074101236251284</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>8.615888052870416</v>
+        <v>9.219419680253136</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>9.1895132982277</v>
+        <v>8.836869918798641</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -3466,11 +3466,11 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6.571268390381882</v>
+        <v>9.203728601212504</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>8.968432028963415</v>
+        <v>8.277714310193796</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3496,7 +3496,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7.701010381259167</v>
+        <v>7.73669294984847</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3511,11 +3511,11 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>8.012986610213169</v>
+        <v>6.679721456274567</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3526,11 +3526,11 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7.016614109579335</v>
+        <v>8.699914105627197</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3541,11 +3541,11 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>9.209446558328624</v>
+        <v>7.001772424285864</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3556,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>7.738665153021669</v>
+        <v>7.655590517725843</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3571,11 +3571,11 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6.684479272625524</v>
+        <v>8.095431324392059</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>
@@ -3586,7 +3586,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>8.944237938456705</v>
+        <v>8.653308070285256</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8.683393886090695</v>
+        <v>9.151066711729356</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3616,7 +3616,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6.847639597883024</v>
+        <v>6.982057944655954</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3631,11 +3631,11 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>9.094937701781554</v>
+        <v>6.726876262956327</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>✅ OK</t>
+          <t>⚠ Below 8 Hrs</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3646,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>7.019495217676577</v>
+        <v>7.936608414826464</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -3661,11 +3661,11 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>7.875926122507204</v>
+        <v>9.472025742594399</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>⚠ Below 8 Hrs</t>
+          <t>✅ OK</t>
         </is>
       </c>
     </row>

</xml_diff>